<commit_message>
[Prerelease v0.1.0dev.5] Spinner loading icon replaced with static icon when animations are disabled. Added asynchronous thumbnail decoding, limited concurrency, and caching per image to reduce UI blocking. Pixel based scrolling implemented, replacing component based scroll. Thumbnail scaling added. Unselect all button added. Keyboard navigation fully implemented.
</commit_message>
<xml_diff>
--- a/docs/Manual-Test-Cases.xlsx
+++ b/docs/Manual-Test-Cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1cd32d6181bdae6/Desktop/Nexmedia-Web-Image-Optimiser/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="179" documentId="8_{C093DD51-22D1-4FD9-815A-E5614C240ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{203D3DB1-D597-44D1-978D-2E678A11C75D}"/>
+  <xr:revisionPtr revIDLastSave="475" documentId="8_{C093DD51-22D1-4FD9-815A-E5614C240ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FB3C41C-8C89-42E5-A086-4B0A887538D0}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2308" uniqueCount="1133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2502" uniqueCount="1152">
   <si>
     <t>Test ID</t>
   </si>
@@ -3419,6 +3419,63 @@
   </si>
   <si>
     <t>Note: clear batch hover styling gets stuck on until a new button is toggled.</t>
+  </si>
+  <si>
+    <t>Fix Needed</t>
+  </si>
+  <si>
+    <t>Failed button style needs to be changed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failure is shown but no information shown. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned size remains native. </t>
+  </si>
+  <si>
+    <t>Export as png and webp both maintain transparency.</t>
+  </si>
+  <si>
+    <t>No "unselect all" functionality. Click and drag scroll is fine, but mousewheel scroll has minor lag.</t>
+  </si>
+  <si>
+    <t>Scrolling is laggy.</t>
+  </si>
+  <si>
+    <t>No degredation observed.</t>
+  </si>
+  <si>
+    <t>Target missed still exportable (correct), failed not exportable (correct).</t>
+  </si>
+  <si>
+    <t>Note: portrait aspect ratios do not display as thumbnails.</t>
+  </si>
+  <si>
+    <t>Simply appends an additional "optimised".</t>
+  </si>
+  <si>
+    <t>Numbers are appended to filename.</t>
+  </si>
+  <si>
+    <t>Keyboard navigation only partially implemented.</t>
+  </si>
+  <si>
+    <t>As before.</t>
+  </si>
+  <si>
+    <t>Launches instantly</t>
+  </si>
+  <si>
+    <t>Windows detects unknown author. AVG antivirus detected but did not block install.</t>
+  </si>
+  <si>
+    <t>Some components do not have focus indicators</t>
+  </si>
+  <si>
+    <t>Issue Fixed?</t>
+  </si>
+  <si>
+    <t>Fix Version</t>
   </si>
 </sst>
 </file>
@@ -3785,11 +3842,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N201"/>
+  <dimension ref="A1:O201"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="27.06640625" customWidth="1"/>
-    <col min="3" max="3" width="35.06640625" customWidth="1"/>
+    <col min="3" max="3" width="49" customWidth="1"/>
     <col min="4" max="4" width="24.3984375" customWidth="1"/>
     <col min="6" max="6" width="67.46484375" customWidth="1"/>
     <col min="7" max="7" width="57.53125" customWidth="1"/>
@@ -3799,9 +3856,11 @@
     <col min="11" max="11" width="10.1328125" customWidth="1"/>
     <col min="12" max="12" width="89" customWidth="1"/>
     <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="14" max="14" width="15.6640625" customWidth="1"/>
+    <col min="15" max="15" width="23.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3841,9 +3900,14 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="N1" s="1" t="s">
+        <v>1150</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>1151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>13</v>
       </c>
@@ -3884,7 +3948,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -3925,7 +3989,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -3966,7 +4030,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -4007,7 +4071,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -4048,7 +4112,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>49</v>
       </c>
@@ -4089,7 +4153,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>54</v>
       </c>
@@ -4130,7 +4194,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>61</v>
       </c>
@@ -4171,7 +4235,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>65</v>
       </c>
@@ -4212,7 +4276,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -4253,7 +4317,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>75</v>
       </c>
@@ -4294,7 +4358,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -4335,7 +4399,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -4376,7 +4440,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -4417,7 +4481,7 @@
         <v>1112</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>100</v>
       </c>
@@ -4896,8 +4960,17 @@
       <c r="I27" t="s">
         <v>156</v>
       </c>
+      <c r="J27" t="s">
+        <v>1110</v>
+      </c>
       <c r="K27" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L27" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M27" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
@@ -8084,8 +8157,17 @@
       <c r="I106" t="s">
         <v>575</v>
       </c>
+      <c r="J106" t="s">
+        <v>1110</v>
+      </c>
       <c r="K106" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L106" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M106" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.45">
@@ -8116,8 +8198,17 @@
       <c r="I107" t="s">
         <v>582</v>
       </c>
+      <c r="J107" t="s">
+        <v>1110</v>
+      </c>
       <c r="K107" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L107" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M107" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.45">
@@ -8148,8 +8239,17 @@
       <c r="I108" t="s">
         <v>588</v>
       </c>
+      <c r="J108" t="s">
+        <v>1110</v>
+      </c>
       <c r="K108" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L108" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M108" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.45">
@@ -8180,8 +8280,17 @@
       <c r="I109" t="s">
         <v>594</v>
       </c>
+      <c r="J109" t="s">
+        <v>1110</v>
+      </c>
       <c r="K109" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L109" t="s">
+        <v>1134</v>
+      </c>
+      <c r="M109" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.45">
@@ -8212,8 +8321,17 @@
       <c r="I110" t="s">
         <v>600</v>
       </c>
+      <c r="J110" t="s">
+        <v>1129</v>
+      </c>
       <c r="K110" t="s">
-        <v>22</v>
+        <v>1133</v>
+      </c>
+      <c r="L110" t="s">
+        <v>1135</v>
+      </c>
+      <c r="M110" t="s">
+        <v>1120</v>
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.45">
@@ -8276,11 +8394,20 @@
       <c r="I112" t="s">
         <v>612</v>
       </c>
+      <c r="J112" t="s">
+        <v>1110</v>
+      </c>
       <c r="K112" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L112" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M112" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="113" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>617</v>
       </c>
@@ -8308,11 +8435,20 @@
       <c r="I113" t="s">
         <v>616</v>
       </c>
+      <c r="J113" t="s">
+        <v>1110</v>
+      </c>
       <c r="K113" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L113" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M113" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>623</v>
       </c>
@@ -8340,11 +8476,20 @@
       <c r="I114" t="s">
         <v>622</v>
       </c>
+      <c r="J114" t="s">
+        <v>1110</v>
+      </c>
       <c r="K114" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L114" t="s">
+        <v>1136</v>
+      </c>
+      <c r="M114" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>627</v>
       </c>
@@ -8372,11 +8517,20 @@
       <c r="I115" t="s">
         <v>626</v>
       </c>
+      <c r="J115" t="s">
+        <v>1110</v>
+      </c>
       <c r="K115" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L115" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M115" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="116" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>633</v>
       </c>
@@ -8404,11 +8558,20 @@
       <c r="I116" t="s">
         <v>632</v>
       </c>
+      <c r="J116" t="s">
+        <v>1110</v>
+      </c>
       <c r="K116" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L116" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M116" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="117" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>639</v>
       </c>
@@ -8436,11 +8599,20 @@
       <c r="I117" t="s">
         <v>638</v>
       </c>
+      <c r="J117" t="s">
+        <v>1110</v>
+      </c>
       <c r="K117" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L117" t="s">
+        <v>1137</v>
+      </c>
+      <c r="M117" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="118" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>645</v>
       </c>
@@ -8472,7 +8644,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>651</v>
       </c>
@@ -8500,11 +8672,20 @@
       <c r="I119" t="s">
         <v>650</v>
       </c>
+      <c r="J119" t="s">
+        <v>1110</v>
+      </c>
       <c r="K119" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L119" t="s">
+        <v>1138</v>
+      </c>
+      <c r="M119" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="120" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>657</v>
       </c>
@@ -8532,11 +8713,20 @@
       <c r="I120" t="s">
         <v>656</v>
       </c>
+      <c r="J120" t="s">
+        <v>1110</v>
+      </c>
       <c r="K120" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L120" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M120" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="121" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>662</v>
       </c>
@@ -8564,11 +8754,20 @@
       <c r="I121" t="s">
         <v>661</v>
       </c>
+      <c r="J121" t="s">
+        <v>1110</v>
+      </c>
       <c r="K121" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L121" t="s">
+        <v>1140</v>
+      </c>
+      <c r="M121" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="122" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>667</v>
       </c>
@@ -8596,11 +8795,20 @@
       <c r="I122" t="s">
         <v>666</v>
       </c>
+      <c r="J122" t="s">
+        <v>1110</v>
+      </c>
       <c r="K122" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L122" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M122" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="123" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>674</v>
       </c>
@@ -8628,11 +8836,20 @@
       <c r="I123" t="s">
         <v>673</v>
       </c>
+      <c r="J123" t="s">
+        <v>1110</v>
+      </c>
       <c r="K123" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L123" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M123" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="124" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>680</v>
       </c>
@@ -8660,11 +8877,20 @@
       <c r="I124" t="s">
         <v>679</v>
       </c>
+      <c r="J124" t="s">
+        <v>1110</v>
+      </c>
       <c r="K124" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L124" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M124" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="125" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>685</v>
       </c>
@@ -8692,11 +8918,20 @@
       <c r="I125" t="s">
         <v>684</v>
       </c>
+      <c r="J125" t="s">
+        <v>1110</v>
+      </c>
       <c r="K125" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L125" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M125" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="126" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>690</v>
       </c>
@@ -8724,11 +8959,20 @@
       <c r="I126" t="s">
         <v>689</v>
       </c>
+      <c r="J126" t="s">
+        <v>1110</v>
+      </c>
       <c r="K126" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L126" t="s">
+        <v>1141</v>
+      </c>
+      <c r="M126" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="127" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>696</v>
       </c>
@@ -8756,11 +9000,20 @@
       <c r="I127" t="s">
         <v>695</v>
       </c>
+      <c r="J127" t="s">
+        <v>1110</v>
+      </c>
       <c r="K127" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L127" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M127" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="128" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>702</v>
       </c>
@@ -8788,11 +9041,20 @@
       <c r="I128" t="s">
         <v>701</v>
       </c>
+      <c r="J128" t="s">
+        <v>1110</v>
+      </c>
       <c r="K128" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L128" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M128" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="129" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>708</v>
       </c>
@@ -8820,11 +9082,20 @@
       <c r="I129" t="s">
         <v>707</v>
       </c>
+      <c r="J129" t="s">
+        <v>1110</v>
+      </c>
       <c r="K129" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L129" t="s">
+        <v>1142</v>
+      </c>
+      <c r="M129" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="130" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>713</v>
       </c>
@@ -8852,11 +9123,20 @@
       <c r="I130" t="s">
         <v>712</v>
       </c>
+      <c r="J130" t="s">
+        <v>1110</v>
+      </c>
       <c r="K130" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L130" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M130" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="131" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>719</v>
       </c>
@@ -8884,11 +9164,20 @@
       <c r="I131" t="s">
         <v>718</v>
       </c>
+      <c r="J131" t="s">
+        <v>1110</v>
+      </c>
       <c r="K131" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L131" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M131" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="132" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>724</v>
       </c>
@@ -8916,11 +9205,20 @@
       <c r="I132" t="s">
         <v>723</v>
       </c>
+      <c r="J132" t="s">
+        <v>1110</v>
+      </c>
       <c r="K132" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L132" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M132" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="133" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>729</v>
       </c>
@@ -8948,11 +9246,20 @@
       <c r="I133" t="s">
         <v>728</v>
       </c>
+      <c r="J133" t="s">
+        <v>1110</v>
+      </c>
       <c r="K133" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L133" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M133" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="134" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>734</v>
       </c>
@@ -8984,7 +9291,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>741</v>
       </c>
@@ -9012,11 +9319,20 @@
       <c r="I135" t="s">
         <v>740</v>
       </c>
+      <c r="J135" t="s">
+        <v>1110</v>
+      </c>
       <c r="K135" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L135" t="s">
+        <v>1143</v>
+      </c>
+      <c r="M135" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="136" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>747</v>
       </c>
@@ -9044,11 +9360,20 @@
       <c r="I136" t="s">
         <v>746</v>
       </c>
+      <c r="J136" t="s">
+        <v>1110</v>
+      </c>
       <c r="K136" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L136" t="s">
+        <v>1144</v>
+      </c>
+      <c r="M136" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="137" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>753</v>
       </c>
@@ -9080,7 +9405,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>759</v>
       </c>
@@ -9108,11 +9433,20 @@
       <c r="I138" t="s">
         <v>758</v>
       </c>
+      <c r="J138" t="s">
+        <v>1110</v>
+      </c>
       <c r="K138" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L138" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M138" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="139" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>763</v>
       </c>
@@ -9140,11 +9474,20 @@
       <c r="I139" t="s">
         <v>762</v>
       </c>
+      <c r="J139" t="s">
+        <v>1110</v>
+      </c>
       <c r="K139" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L139" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M139" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="140" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>767</v>
       </c>
@@ -9172,11 +9515,20 @@
       <c r="I140" t="s">
         <v>766</v>
       </c>
+      <c r="J140" t="s">
+        <v>1110</v>
+      </c>
       <c r="K140" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L140" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M140" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="141" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>774</v>
       </c>
@@ -9204,11 +9556,20 @@
       <c r="I141" t="s">
         <v>773</v>
       </c>
+      <c r="J141" t="s">
+        <v>1110</v>
+      </c>
       <c r="K141" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L141" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M141" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="142" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>780</v>
       </c>
@@ -9240,7 +9601,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>786</v>
       </c>
@@ -9272,7 +9633,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>791</v>
       </c>
@@ -9300,11 +9661,20 @@
       <c r="I144" t="s">
         <v>790</v>
       </c>
+      <c r="J144" t="s">
+        <v>1110</v>
+      </c>
       <c r="K144" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L144" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M144" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="145" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>797</v>
       </c>
@@ -9332,11 +9702,20 @@
       <c r="I145" t="s">
         <v>796</v>
       </c>
+      <c r="J145" t="s">
+        <v>1110</v>
+      </c>
       <c r="K145" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L145" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M145" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="146" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>803</v>
       </c>
@@ -9368,7 +9747,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>809</v>
       </c>
@@ -9396,11 +9775,20 @@
       <c r="I147" t="s">
         <v>808</v>
       </c>
+      <c r="J147" t="s">
+        <v>1110</v>
+      </c>
       <c r="K147" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L147" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M147" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="148" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>815</v>
       </c>
@@ -9428,11 +9816,20 @@
       <c r="I148" t="s">
         <v>814</v>
       </c>
+      <c r="J148" t="s">
+        <v>1110</v>
+      </c>
       <c r="K148" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L148" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M148" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="149" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>821</v>
       </c>
@@ -9464,7 +9861,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>826</v>
       </c>
@@ -9496,7 +9893,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>831</v>
       </c>
@@ -9524,11 +9921,20 @@
       <c r="I151" t="s">
         <v>830</v>
       </c>
+      <c r="J151" t="s">
+        <v>1110</v>
+      </c>
       <c r="K151" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L151" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M151" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="152" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>834</v>
       </c>
@@ -9556,11 +9962,20 @@
       <c r="I152" t="s">
         <v>833</v>
       </c>
+      <c r="J152" t="s">
+        <v>1110</v>
+      </c>
       <c r="K152" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L152" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M152" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="153" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>840</v>
       </c>
@@ -9592,7 +10007,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>845</v>
       </c>
@@ -9624,7 +10039,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>850</v>
       </c>
@@ -9656,7 +10071,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>856</v>
       </c>
@@ -9688,7 +10103,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>862</v>
       </c>
@@ -9720,7 +10135,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>868</v>
       </c>
@@ -9752,7 +10167,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>875</v>
       </c>
@@ -9784,7 +10199,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>880</v>
       </c>
@@ -9816,7 +10231,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>887</v>
       </c>
@@ -9848,7 +10263,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>893</v>
       </c>
@@ -9880,7 +10295,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>899</v>
       </c>
@@ -9912,7 +10327,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>904</v>
       </c>
@@ -9944,7 +10359,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>909</v>
       </c>
@@ -9976,7 +10391,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>915</v>
       </c>
@@ -10008,7 +10423,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>920</v>
       </c>
@@ -10040,7 +10455,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>925</v>
       </c>
@@ -10072,7 +10487,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>931</v>
       </c>
@@ -10104,7 +10519,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>936</v>
       </c>
@@ -10136,7 +10551,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>942</v>
       </c>
@@ -10168,7 +10583,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>948</v>
       </c>
@@ -10200,7 +10615,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>954</v>
       </c>
@@ -10232,7 +10647,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>960</v>
       </c>
@@ -10264,7 +10679,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>967</v>
       </c>
@@ -10292,11 +10707,20 @@
       <c r="I175" t="s">
         <v>966</v>
       </c>
+      <c r="J175" t="s">
+        <v>1110</v>
+      </c>
       <c r="K175" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L175" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M175" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="176" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>973</v>
       </c>
@@ -10324,11 +10748,20 @@
       <c r="I176" t="s">
         <v>972</v>
       </c>
+      <c r="J176" t="s">
+        <v>1110</v>
+      </c>
       <c r="K176" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L176" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M176" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="177" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>977</v>
       </c>
@@ -10356,11 +10789,20 @@
       <c r="I177" t="s">
         <v>976</v>
       </c>
+      <c r="J177" t="s">
+        <v>1110</v>
+      </c>
       <c r="K177" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L177" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M177" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="178" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>982</v>
       </c>
@@ -10388,11 +10830,20 @@
       <c r="I178" t="s">
         <v>981</v>
       </c>
+      <c r="J178" t="s">
+        <v>1110</v>
+      </c>
       <c r="K178" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L178" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M178" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="179" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>988</v>
       </c>
@@ -10420,11 +10871,20 @@
       <c r="I179" t="s">
         <v>987</v>
       </c>
+      <c r="J179" t="s">
+        <v>1110</v>
+      </c>
       <c r="K179" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L179" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M179" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="180" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>994</v>
       </c>
@@ -10452,11 +10912,20 @@
       <c r="I180" t="s">
         <v>993</v>
       </c>
+      <c r="J180" t="s">
+        <v>1110</v>
+      </c>
       <c r="K180" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L180" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M180" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="181" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>1000</v>
       </c>
@@ -10484,11 +10953,20 @@
       <c r="I181" t="s">
         <v>999</v>
       </c>
+      <c r="J181" t="s">
+        <v>1110</v>
+      </c>
       <c r="K181" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L181" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M181" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="182" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>1006</v>
       </c>
@@ -10516,11 +10994,20 @@
       <c r="I182" t="s">
         <v>1005</v>
       </c>
+      <c r="J182" t="s">
+        <v>1129</v>
+      </c>
       <c r="K182" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1133</v>
+      </c>
+      <c r="L182" t="s">
+        <v>1145</v>
+      </c>
+      <c r="M182" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="183" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>1011</v>
       </c>
@@ -10548,11 +11035,20 @@
       <c r="I183" t="s">
         <v>1010</v>
       </c>
+      <c r="J183" t="s">
+        <v>1129</v>
+      </c>
       <c r="K183" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1133</v>
+      </c>
+      <c r="L183" t="s">
+        <v>1146</v>
+      </c>
+      <c r="M183" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="184" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>1016</v>
       </c>
@@ -10580,11 +11076,20 @@
       <c r="I184" t="s">
         <v>1015</v>
       </c>
+      <c r="J184" t="s">
+        <v>1129</v>
+      </c>
       <c r="K184" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1133</v>
+      </c>
+      <c r="L184" t="s">
+        <v>1149</v>
+      </c>
+      <c r="M184" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="185" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>1021</v>
       </c>
@@ -10612,11 +11117,20 @@
       <c r="I185" t="s">
         <v>1020</v>
       </c>
+      <c r="J185" t="s">
+        <v>1110</v>
+      </c>
       <c r="K185" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L185" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M185" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="186" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>1025</v>
       </c>
@@ -10644,11 +11158,20 @@
       <c r="I186" t="s">
         <v>1024</v>
       </c>
+      <c r="J186" t="s">
+        <v>1110</v>
+      </c>
       <c r="K186" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L186" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M186" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="187" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>1032</v>
       </c>
@@ -10676,11 +11199,20 @@
       <c r="I187" t="s">
         <v>1031</v>
       </c>
+      <c r="J187" t="s">
+        <v>1110</v>
+      </c>
       <c r="K187" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L187" t="s">
+        <v>1147</v>
+      </c>
+      <c r="M187" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="188" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>1037</v>
       </c>
@@ -10708,11 +11240,20 @@
       <c r="I188" t="s">
         <v>1036</v>
       </c>
+      <c r="J188" t="s">
+        <v>1110</v>
+      </c>
       <c r="K188" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L188" t="s">
+        <v>1147</v>
+      </c>
+      <c r="M188" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="189" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>1041</v>
       </c>
@@ -10740,11 +11281,20 @@
       <c r="I189" t="s">
         <v>1040</v>
       </c>
+      <c r="J189" t="s">
+        <v>1110</v>
+      </c>
       <c r="K189" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L189" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M189" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="190" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>1047</v>
       </c>
@@ -10772,11 +11322,20 @@
       <c r="I190" t="s">
         <v>1046</v>
       </c>
+      <c r="J190" t="s">
+        <v>1110</v>
+      </c>
       <c r="K190" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L190" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M190" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="191" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>1052</v>
       </c>
@@ -10804,11 +11363,20 @@
       <c r="I191" t="s">
         <v>1051</v>
       </c>
+      <c r="J191" t="s">
+        <v>1110</v>
+      </c>
       <c r="K191" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L191" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M191" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="192" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>1058</v>
       </c>
@@ -10836,11 +11404,20 @@
       <c r="I192" t="s">
         <v>1057</v>
       </c>
+      <c r="J192" t="s">
+        <v>1110</v>
+      </c>
       <c r="K192" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L192" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M192" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="193" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>1064</v>
       </c>
@@ -10868,11 +11445,20 @@
       <c r="I193" t="s">
         <v>1063</v>
       </c>
+      <c r="J193" t="s">
+        <v>1110</v>
+      </c>
       <c r="K193" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L193" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M193" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="194" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>1069</v>
       </c>
@@ -10904,7 +11490,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>1074</v>
       </c>
@@ -10932,11 +11518,20 @@
       <c r="I195" t="s">
         <v>1073</v>
       </c>
+      <c r="J195" t="s">
+        <v>1110</v>
+      </c>
       <c r="K195" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L195" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M195" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="196" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>1079</v>
       </c>
@@ -10964,11 +11559,20 @@
       <c r="I196" t="s">
         <v>1078</v>
       </c>
+      <c r="J196" t="s">
+        <v>1110</v>
+      </c>
       <c r="K196" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L196" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M196" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="197" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>1086</v>
       </c>
@@ -10996,11 +11600,20 @@
       <c r="I197" t="s">
         <v>1085</v>
       </c>
+      <c r="J197" t="s">
+        <v>1129</v>
+      </c>
       <c r="K197" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L197" t="s">
+        <v>1148</v>
+      </c>
+      <c r="M197" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="198" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>1092</v>
       </c>
@@ -11028,11 +11641,20 @@
       <c r="I198" t="s">
         <v>1091</v>
       </c>
+      <c r="J198" t="s">
+        <v>1110</v>
+      </c>
       <c r="K198" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L198" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M198" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="199" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>1098</v>
       </c>
@@ -11064,7 +11686,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>1104</v>
       </c>
@@ -11092,11 +11714,20 @@
       <c r="I200" t="s">
         <v>1103</v>
       </c>
+      <c r="J200" t="s">
+        <v>1110</v>
+      </c>
       <c r="K200" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.45">
+        <v>1113</v>
+      </c>
+      <c r="L200" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M200" t="s">
+        <v>1120</v>
+      </c>
+    </row>
+    <row r="201" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>1114</v>
       </c>
@@ -11124,8 +11755,17 @@
       <c r="I201" t="s">
         <v>1109</v>
       </c>
+      <c r="J201" t="s">
+        <v>1110</v>
+      </c>
       <c r="K201" t="s">
-        <v>22</v>
+        <v>1113</v>
+      </c>
+      <c r="L201" t="s">
+        <v>1111</v>
+      </c>
+      <c r="M201" t="s">
+        <v>1120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>